<commit_message>
Add subscription import and prorated uninvoiced revenue tracking.
Extend Excel import to create plans and subscriptions from cost and date columns. Count uninvoiced subscription value as revenue spread across the subscription period, shown alongside invoice payments on the dashboard.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/public/templates/membri-template.xlsx
+++ b/public/templates/membri-template.xlsx
@@ -60,9 +60,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:J4"/>
   <sheetData>
-    <row r="1" spans="1:6" customHeight="0">
+    <row r="1" spans="1:10" customHeight="0">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>Prenume</t>
@@ -90,11 +90,31 @@
       </c>
       <c r="F1" s="0" t="inlineStr">
         <is>
+          <t>Abonament</t>
+        </is>
+      </c>
+      <c r="G1" s="0" t="inlineStr">
+        <is>
+          <t>Cost</t>
+        </is>
+      </c>
+      <c r="H1" s="0" t="inlineStr">
+        <is>
+          <t>Data start</t>
+        </is>
+      </c>
+      <c r="I1" s="0" t="inlineStr">
+        <is>
+          <t>Data expirare</t>
+        </is>
+      </c>
+      <c r="J1" s="0" t="inlineStr">
+        <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="2" spans="1:6" customHeight="0">
+    <row r="2" spans="1:10" customHeight="0">
       <c r="A2" s="0" t="inlineStr">
         <is>
           <t>Andrei</t>
@@ -122,11 +142,31 @@
       </c>
       <c r="F2" s="0" t="inlineStr">
         <is>
+          <t>Lunar</t>
+        </is>
+      </c>
+      <c r="G2" s="0" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="H2" s="0" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="I2" s="0" t="inlineStr">
+        <is>
+          <t>01/07/2026</t>
+        </is>
+      </c>
+      <c r="J2" s="0" t="inlineStr">
+        <is>
           <t>Abonament anual</t>
         </is>
       </c>
     </row>
-    <row r="3" spans="1:6" customHeight="0">
+    <row r="3" spans="1:10" customHeight="0">
       <c r="A3" s="0" t="inlineStr">
         <is>
           <t>Maria</t>
@@ -152,8 +192,28 @@
           <t>22/07/1985</t>
         </is>
       </c>
-    </row>
-    <row r="4" spans="1:6" customHeight="0">
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t>Trimestrial</t>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t>01/06/2026</t>
+        </is>
+      </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t>01/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:10" customHeight="0">
       <c r="A4" s="0" t="inlineStr">
         <is>
           <t>George</t>
@@ -180,6 +240,16 @@
         </is>
       </c>
       <c r="F4" s="0" t="inlineStr">
+        <is>
+          <t>Lunar</t>
+        </is>
+      </c>
+      <c r="G4" s="0" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="J4" s="0" t="inlineStr">
         <is>
           <t>Preferă antrenament dimineața</t>
         </is>

</xml_diff>